<commit_message>
Refine feature gap analysis and documentation updates
- Enhanced descriptions for features in the Features Map to clarify buyer relevance and evidence status.
- Updated funding feature description to specify matching criteria and saturation levels.
- Revised customer management, fundraising management, and growth management entries to reflect detailed insights from research phases.
- Consolidated investor due diligence and investment management features, emphasizing buyer distinctions.
- Adjusted portfolio dashboard and startup performance dashboard entries for clarity on market standards.
- Updated exported timestamps in JSON files for consistency across datasets.
- Modified Python scripts to improve documentation generation and feature mapping accuracy.
</commit_message>
<xml_diff>
--- a/docs/research/_exports/xlsx/10_Feature_Gap.xlsx
+++ b/docs/research/_exports/xlsx/10_Feature_Gap.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="687" uniqueCount="418">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="687" uniqueCount="421">
   <si>
     <t>The Six Differentiators</t>
   </si>
@@ -810,96 +810,126 @@
     <t>Customer Management</t>
   </si>
   <si>
-    <t>No evidence. Founder-side.</t>
+    <t>Startup-side CRM for customer discovery, retention and churn. No evidence in any phase, no competitor demand, and it belongs to the founder's business rather than the institutional buyer this product sells to.</t>
   </si>
   <si>
     <t>Funding</t>
   </si>
   <si>
-    <t>Scheme-eligibility matching is the second half of differentiator 1. A plain grant LIST is saturated (11 of 40 native) - matching is not.</t>
+    <t>Scheme-eligibility matching is the second half of differentiator 1. A plain grant LIST is saturated at 11 of 40 native - matching a venture's TRL and sector against actual scheme criteria is not built by anyone.</t>
   </si>
   <si>
     <t>Fundraising Management</t>
   </si>
   <si>
+    <t>Investor-side: pipeline, data rooms, term sheets, cap table. Phase 9 found Startup India Hub and MAARG already overlapping this, and it addresses the investor rather than the university that StartupHub sells to.</t>
+  </si>
+  <si>
+    <t>Growth Management</t>
+  </si>
+  <si>
+    <t>Startup-side growth planning and metrics. Nothing in eleven phases evidences demand, and the buyer who would pay for it is the founder, who is not in the procurement chain Phase 2 mapped.</t>
+  </si>
+  <si>
+    <t>Startup Performance Dashboard</t>
+  </si>
+  <si>
+    <t>28 of 40 vendors build reporting natively or better and 27 build analytics. Rule 1 applies: this cannot be a differentiator and must not appear in positioning. It remains a v1 parity requirement.</t>
+  </si>
+  <si>
+    <t>Risk Management</t>
+  </si>
+  <si>
+    <t>Plausible and connected to the TRL object, but Phase 11 found no user asking for risk scoring. Cannot be scoped without interviews.</t>
+  </si>
+  <si>
+    <t>Founder AI Assistant</t>
+  </si>
+  <si>
+    <t>CONTRADICTED</t>
+  </si>
+  <si>
+    <t>Phase 11: zero users asked for AI, and 'AI assistant' is exactly the positioning Phase 11 declined to make. Keep as an internal surface over the TRL object, never as a differentiator.</t>
+  </si>
+  <si>
+    <t>Incubator / Accelerator (portfolio)</t>
+  </si>
+  <si>
+    <t>Portfolio view is standard in 15+ vendors.</t>
+  </si>
+  <si>
+    <t>Program Management</t>
+  </si>
+  <si>
+    <t>Cohort and programme management is the most built capability in the category.</t>
+  </si>
+  <si>
+    <t>Portfolio Dashboard</t>
+  </si>
+  <si>
+    <t>The at-a-glance cohort table with stage, risk and progress is standard in every vendor with a portfolio view. Fifteen or more build it natively. Keep it for parity; never sell it.</t>
+  </si>
+  <si>
+    <t>Investor Due Diligence</t>
+  </si>
+  <si>
+    <t>The diligence workspace and data room serve the investor's due-diligence process, not the university's innovation return. Phase 9 found no named Indian university asking for it.</t>
+  </si>
+  <si>
+    <t>Investment Management</t>
+  </si>
+  <si>
+    <t>Post-investment portfolio tracking for funds. A different buyer, a different budget and a different approval chain entirely from the IIC coordinator.</t>
+  </si>
+  <si>
+    <t>Resource Provider</t>
+  </si>
+  <si>
+    <t>Marketplace supply side: cloud credits, labs, hardware, consultants. Only 3 of 40 vendors build resource management natively, so the gap is real - but Phase 5 concluded we should not compete here.</t>
+  </si>
+  <si>
+    <t>Corporate Pilot Management</t>
+  </si>
+  <si>
+    <t>Challenge-to-pilot-to-contract workflow. corporate_match is 5 native and 18 partial across the market - mostly weak, and there is no evidence in any phase that the university buyer wants it inside the v1 system of record.</t>
+  </si>
+  <si>
+    <t>Talent / Professional</t>
+  </si>
+  <si>
+    <t>Marketplace supply side for skills and freelancing. Two-sided marketplace economics with no demand evidence and no institutional buyer attached.</t>
+  </si>
+  <si>
+    <t>Notification &amp; Alert Engine</t>
+  </si>
+  <si>
+    <t>Centralised alerts are standard across the category. Phase 11's one real complaint in this area was email reaching spam - a deliverability problem, not a missing feature. Building an engine against it solves the wrong thing.</t>
+  </si>
+  <si>
+    <t>Incubator Resource Management</t>
+  </si>
+  <si>
+    <t>Same reasoning as #8 - real gap, wrong strategic choice.</t>
+  </si>
+  <si>
+    <t>Mentor / Expert</t>
+  </si>
+  <si>
+    <t>Retained only for the NDA-tiered visibility half (GAP-07).</t>
+  </si>
+  <si>
+    <t>IPR / Legal Professional</t>
+  </si>
+  <si>
+    <t>Second persona for differentiator 2; expand after the venture record ships.</t>
+  </si>
+  <si>
+    <t>Investor</t>
+  </si>
+  <si>
     <t>Investor-side. Not this buyer.</t>
   </si>
   <si>
-    <t>Growth Management</t>
-  </si>
-  <si>
-    <t>Startup-side. No evidence.</t>
-  </si>
-  <si>
-    <t>Startup Performance Dashboard</t>
-  </si>
-  <si>
-    <t>28 of 40 build reporting, 27 analytics. Rule 1 retires this as a differentiator.</t>
-  </si>
-  <si>
-    <t>Risk Management</t>
-  </si>
-  <si>
-    <t>Plausible and connected to the TRL object, but Phase 11 found no user asking for risk scoring. Cannot be scoped without interviews.</t>
-  </si>
-  <si>
-    <t>Founder AI Assistant</t>
-  </si>
-  <si>
-    <t>CONTRADICTED</t>
-  </si>
-  <si>
-    <t>Phase 11: zero users asked for AI, and 'AI assistant' is exactly the positioning Phase 11 declined to make. Keep as an internal surface over the TRL object, never as a differentiator.</t>
-  </si>
-  <si>
-    <t>Incubator / Accelerator (portfolio)</t>
-  </si>
-  <si>
-    <t>Portfolio view is standard in 15+ vendors.</t>
-  </si>
-  <si>
-    <t>Program Management</t>
-  </si>
-  <si>
-    <t>Cohort and programme management is the most built capability in the category.</t>
-  </si>
-  <si>
-    <t>Portfolio Dashboard</t>
-  </si>
-  <si>
-    <t>See #16.</t>
-  </si>
-  <si>
-    <t>Incubator Resource Management</t>
-  </si>
-  <si>
-    <t>Same reasoning as #8 - real gap, wrong strategic choice.</t>
-  </si>
-  <si>
-    <t>Mentor / Expert</t>
-  </si>
-  <si>
-    <t>Retained only for the NDA-tiered visibility half (GAP-07).</t>
-  </si>
-  <si>
-    <t>IPR / Legal Professional</t>
-  </si>
-  <si>
-    <t>Second persona for differentiator 2; expand after the venture record ships.</t>
-  </si>
-  <si>
-    <t>Investor</t>
-  </si>
-  <si>
-    <t>Investor Due Diligence</t>
-  </si>
-  <si>
-    <t>Investor-side.</t>
-  </si>
-  <si>
-    <t>Investment Management</t>
-  </si>
-  <si>
     <t>Government / Institution</t>
   </si>
   <si>
@@ -912,12 +942,6 @@
     <t>Same object as differentiator 1's scheme mapping, seen from the government side.</t>
   </si>
   <si>
-    <t>Resource Provider</t>
-  </si>
-  <si>
-    <t>Marketplace-side.</t>
-  </si>
-  <si>
     <t>Resource Marketplace</t>
   </si>
   <si>
@@ -930,21 +954,12 @@
     <t>Phase 9 found corporate_match is 5 native / 18 partial - mostly weak. No evidence the university buyer wants this in v1.</t>
   </si>
   <si>
-    <t>Corporate Pilot Management</t>
-  </si>
-  <si>
-    <t>Same reasoning as #32.</t>
-  </si>
-  <si>
     <t>University / Research Institution</t>
   </si>
   <si>
     <t>This IS the buyer. Research-to-IP-to-startup connection is differentiator 2.</t>
   </si>
   <si>
-    <t>Talent / Professional</t>
-  </si>
-  <si>
     <t>StartupHub Admin</t>
   </si>
   <si>
@@ -967,12 +982,6 @@
   </si>
   <si>
     <t>Needed eventually, not differentiating, and heavily commoditised.</t>
-  </si>
-  <si>
-    <t>Notification &amp; Alert Engine</t>
-  </si>
-  <si>
-    <t>Standard across the category.</t>
   </si>
   <si>
     <t>The Central AI Engine</t>
@@ -4385,7 +4394,7 @@
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="5">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>279</v>
@@ -4399,7 +4408,7 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="5">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>281</v>
@@ -4413,7 +4422,7 @@
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="5">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>283</v>
@@ -4427,7 +4436,7 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="5">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>285</v>
@@ -4436,217 +4445,217 @@
         <v>241</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>263</v>
+        <v>286</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="5">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C30" s="9" t="s">
         <v>241</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="5">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="5">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>289</v>
-      </c>
-      <c r="C32" s="8" t="s">
-        <v>236</v>
+        <v>291</v>
+      </c>
+      <c r="C32" s="9" t="s">
+        <v>241</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="5">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>291</v>
-      </c>
-      <c r="C33" s="8" t="s">
-        <v>236</v>
+        <v>293</v>
+      </c>
+      <c r="C33" s="9" t="s">
+        <v>241</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="5">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C34" s="9" t="s">
         <v>241</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="5">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C35" s="9" t="s">
         <v>241</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="5">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>297</v>
-      </c>
-      <c r="C36" s="9" t="s">
-        <v>241</v>
+        <v>299</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>236</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="5">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>299</v>
-      </c>
-      <c r="C37" s="9" t="s">
-        <v>241</v>
+        <v>301</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>236</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="5">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>301</v>
-      </c>
-      <c r="C38" s="8" t="s">
-        <v>236</v>
+        <v>303</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>241</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="5">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="C39" s="9" t="s">
         <v>241</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>294</v>
+        <v>306</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="5">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="C40" s="8" t="s">
         <v>236</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="5">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="C41" s="8" t="s">
         <v>236</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="5">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>308</v>
-      </c>
-      <c r="C42" s="9" t="s">
-        <v>244</v>
+        <v>311</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>236</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="5">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="5">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="C44" s="9" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -4654,13 +4663,13 @@
         <v>41</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="C45" s="6" t="s">
         <v>271</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -4668,13 +4677,13 @@
         <v>42</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="C46" s="7" t="s">
         <v>233</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -4682,13 +4691,13 @@
         <v>43</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="C47" s="7" t="s">
         <v>233</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -4696,13 +4705,13 @@
         <v>44</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="C48" s="7" t="s">
         <v>233</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -4710,13 +4719,13 @@
         <v>45</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="C49" s="7" t="s">
         <v>233</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -4724,13 +4733,13 @@
         <v>46</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="C50" s="8" t="s">
         <v>236</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
     </row>
   </sheetData>
@@ -4752,194 +4761,194 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="30" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="30" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>90</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="5" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>236</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="5" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>244</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="5" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>236</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="5" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="B8" s="9" t="s">
         <v>241</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="5" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="B9" s="9" t="s">
         <v>241</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="5" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="B10" s="9" t="s">
         <v>241</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="5" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="B11" s="8" t="s">
         <v>236</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="5" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="B12" s="9" t="s">
         <v>244</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="5" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="B13" s="9" t="s">
         <v>241</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="5" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="B14" s="9" t="s">
         <v>244</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="5" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>271</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="5" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="B16" s="8" t="s">
         <v>236</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
   </sheetData>
@@ -4961,86 +4970,86 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="30" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="30" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="5" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="B5" s="5"/>
       <c r="C5" s="5" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="5" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="5" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="5" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="5" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="5" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="B8" s="5"/>
       <c r="C8" s="5" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="5" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="B9" s="5"/>
       <c r="C9" s="5" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
     </row>
   </sheetData>
@@ -5062,34 +5071,34 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="30" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="30" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="5" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="B5" s="5">
         <v>28</v>
@@ -5101,12 +5110,12 @@
         <v>0.7</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="5" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="B6" s="5">
         <v>27</v>
@@ -5118,12 +5127,12 @@
         <v>0.675</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="5" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="B7" s="5">
         <v>21</v>
@@ -5135,12 +5144,12 @@
         <v>0.525</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="5" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="B8" s="5">
         <v>20</v>
@@ -5152,12 +5161,12 @@
         <v>0.5</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="5" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="B9" s="5">
         <v>15</v>
@@ -5169,7 +5178,7 @@
         <v>0.375</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -5186,12 +5195,12 @@
         <v>0.275</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="5" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="B11" s="5">
         <v>10</v>
@@ -5203,12 +5212,12 @@
         <v>0.25</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="5" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="B12" s="5">
         <v>9</v>
@@ -5220,7 +5229,7 @@
         <v>0.225</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -5237,12 +5246,12 @@
         <v>0.175</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="5" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="B14" s="5">
         <v>7</v>
@@ -5254,12 +5263,12 @@
         <v>0.175</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="5" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="B15" s="5">
         <v>7</v>
@@ -5271,12 +5280,12 @@
         <v>0.175</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="5" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="B16" s="5">
         <v>5</v>
@@ -5288,7 +5297,7 @@
         <v>0.125</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -5305,12 +5314,12 @@
         <v>0.075</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="5" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="B18" s="5">
         <v>3</v>
@@ -5322,12 +5331,12 @@
         <v>0.075</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="5" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="B19" s="5">
         <v>2</v>
@@ -5339,7 +5348,7 @@
         <v>0.05</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
     </row>
   </sheetData>
@@ -5361,34 +5370,34 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="30" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="30" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>14</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="5" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>19</v>
@@ -5400,12 +5409,12 @@
         <v>25</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="5" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>30</v>
@@ -5417,12 +5426,12 @@
         <v>36</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="5" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>41</v>
@@ -5434,12 +5443,12 @@
         <v>25</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="5" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>51</v>
@@ -5451,12 +5460,12 @@
         <v>56</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="5" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>61</v>
@@ -5468,12 +5477,12 @@
         <v>66</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="5" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="B10" s="5" t="s">
         <v>71</v>
@@ -5485,7 +5494,7 @@
         <v>56</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
     </row>
   </sheetData>

</xml_diff>